<commit_message>
Added stan files, new modelling framework, new correlation results, niche breadth and density data, also lot more collaborator comparisons
</commit_message>
<xml_diff>
--- a/data/Collaborator data/NJ_ bulbuls/Morphometrics of Thapsinillas (all specimens).xlsx
+++ b/data/Collaborator data/NJ_ bulbuls/Morphometrics of Thapsinillas (all specimens).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/brinda/Documents/MRes project/data/Collaborator data/NJ_ bulbuls/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{586DC240-09E4-A14E-91FD-9BA48DF76938}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E2B4B12-B6C7-FB46-BE0B-C367FDDD1924}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1820" yWindow="500" windowWidth="28840" windowHeight="16320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -997,6 +997,7 @@
   <dimension ref="A1:S135"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
+    <col min="1" max="1" width="27" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
     <col min="3" max="3" width="7.1640625" customWidth="1"/>
     <col min="4" max="4" width="14" customWidth="1"/>

</xml_diff>